<commit_message>
#13 JLCPCB and LCSC BOM Completed
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/LCSC BOM-John.xlsx
+++ b/Deliverables/BOM/LCSC BOM-John.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="315">
   <si>
     <t>Component list</t>
   </si>
@@ -942,19 +942,28 @@
     <t>Digikey</t>
   </si>
   <si>
-    <t>QM3001K-VB</t>
-  </si>
-  <si>
-    <t>C725140</t>
-  </si>
-  <si>
-    <t>NON Stock On LCSC</t>
-  </si>
-  <si>
     <t>STMicroelectronics</t>
   </si>
   <si>
-    <t>C2053863</t>
+    <t>DMP3099L-7-VB</t>
+  </si>
+  <si>
+    <t>C558116</t>
+  </si>
+  <si>
+    <t>STM32F070CBT6</t>
+  </si>
+  <si>
+    <t>C74909</t>
+  </si>
+  <si>
+    <t>PSPMAA0503-2R2M-ANP</t>
+  </si>
+  <si>
+    <t>C436533</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YE Part Design me Change hoga Is ka footprint Change ha </t>
   </si>
 </sst>
 </file>
@@ -1494,7 +1503,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1731,6 +1740,15 @@
     <xf numFmtId="0" fontId="20" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="23" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2090,7 +2108,7 @@
     <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="16.5703125" bestFit="1" customWidth="1"/>
@@ -3457,7 +3475,7 @@
       <c r="R29" s="51"/>
       <c r="S29" s="59"/>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" ht="36" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="46">
         <f>ROW(B30) - ROW($B$9)</f>
@@ -3475,14 +3493,18 @@
       <c r="F30" s="37" t="s">
         <v>235</v>
       </c>
-      <c r="G30" s="37" t="s">
+      <c r="G30" s="66" t="s">
         <v>116</v>
       </c>
       <c r="H30" s="37" t="s">
         <v>170</v>
       </c>
-      <c r="I30" s="37"/>
-      <c r="J30" s="37"/>
+      <c r="I30" s="37" t="s">
+        <v>312</v>
+      </c>
+      <c r="J30" s="37" t="s">
+        <v>313</v>
+      </c>
       <c r="K30" s="37" t="s">
         <v>246</v>
       </c>
@@ -3494,19 +3516,21 @@
         <v>50</v>
       </c>
       <c r="N30" s="37">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="O30" s="65" t="s">
-        <v>306</v>
+        <v>240</v>
       </c>
       <c r="P30" s="38">
-        <v>1.2</v>
+        <v>0.11509999999999999</v>
       </c>
       <c r="Q30" s="38">
         <f>P30*N30</f>
-        <v>72</v>
-      </c>
-      <c r="R30" s="37"/>
+        <v>6.3304999999999998</v>
+      </c>
+      <c r="R30" s="73" t="s">
+        <v>314</v>
+      </c>
       <c r="S30" s="59"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
@@ -3533,8 +3557,12 @@
       <c r="H31" s="51" t="s">
         <v>171</v>
       </c>
-      <c r="I31" s="51"/>
-      <c r="J31" s="51"/>
+      <c r="I31" s="51" t="s">
+        <v>246</v>
+      </c>
+      <c r="J31" s="51" t="s">
+        <v>246</v>
+      </c>
       <c r="K31" s="51" t="s">
         <v>246</v>
       </c>
@@ -3586,10 +3614,10 @@
         <v>172</v>
       </c>
       <c r="I32" s="37" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J32" s="37" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K32" s="63" t="s">
         <v>246</v>
@@ -3602,21 +3630,19 @@
         <v>50</v>
       </c>
       <c r="N32" s="37">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="O32" s="65" t="s">
         <v>240</v>
       </c>
       <c r="P32" s="38">
-        <v>0.2</v>
+        <v>7.4399999999999994E-2</v>
       </c>
       <c r="Q32" s="38">
         <f>P32*N32</f>
-        <v>12</v>
-      </c>
-      <c r="R32" s="73" t="s">
-        <v>309</v>
-      </c>
+        <v>4.0919999999999996</v>
+      </c>
+      <c r="R32" s="73"/>
       <c r="S32" s="59"/>
     </row>
     <row r="33" spans="1:19" ht="84" x14ac:dyDescent="0.25">
@@ -4627,8 +4653,8 @@
       <c r="R50" s="51"/>
       <c r="S50" s="59"/>
     </row>
-    <row r="51" spans="1:19" ht="36" x14ac:dyDescent="0.25">
-      <c r="A51" s="1"/>
+    <row r="51" spans="1:19" s="87" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A51" s="85"/>
       <c r="B51" s="46">
         <f>ROW(B51) - ROW($B$9)</f>
         <v>42</v>
@@ -4670,7 +4696,7 @@
       <c r="N51" s="37">
         <v>52</v>
       </c>
-      <c r="O51" s="65" t="s">
+      <c r="O51" s="86" t="s">
         <v>240</v>
       </c>
       <c r="P51" s="38">
@@ -4813,14 +4839,14 @@
       <c r="F54" s="62" t="s">
         <v>238</v>
       </c>
-      <c r="G54" s="51" t="s">
+      <c r="G54" s="67" t="s">
         <v>125</v>
       </c>
       <c r="H54" s="51" t="s">
+        <v>307</v>
+      </c>
+      <c r="I54" s="51" t="s">
         <v>310</v>
-      </c>
-      <c r="I54" s="51" t="s">
-        <v>246</v>
       </c>
       <c r="J54" s="51" t="s">
         <v>311</v>
@@ -4842,15 +4868,13 @@
         <v>240</v>
       </c>
       <c r="P54" s="52">
-        <v>7.7206999999999999</v>
+        <v>1.4335</v>
       </c>
       <c r="Q54" s="52">
         <f t="shared" ref="Q54" si="24">P54*N54</f>
-        <v>401.47640000000001</v>
-      </c>
-      <c r="R54" s="74" t="s">
-        <v>309</v>
-      </c>
+        <v>74.542000000000002</v>
+      </c>
+      <c r="R54" s="74"/>
       <c r="S54" s="59"/>
     </row>
     <row r="55" spans="1:19" ht="36" x14ac:dyDescent="0.25">
@@ -5042,7 +5066,7 @@
       <c r="P58" s="84"/>
       <c r="Q58" s="48">
         <f>SUM(Q10:Q57)</f>
-        <v>1052.9630999999999</v>
+        <v>652.45119999999997</v>
       </c>
       <c r="R58" s="79"/>
       <c r="S58" s="80"/>
@@ -5068,7 +5092,7 @@
       <c r="P59" s="84"/>
       <c r="Q59" s="49">
         <f>Q58/50</f>
-        <v>21.059262</v>
+        <v>13.049023999999999</v>
       </c>
       <c r="R59" s="81"/>
       <c r="S59" s="82"/>
@@ -5083,52 +5107,52 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O11" r:id="rId1"/>
-    <hyperlink ref="O12" r:id="rId2"/>
-    <hyperlink ref="O13" r:id="rId3"/>
-    <hyperlink ref="O14" r:id="rId4"/>
-    <hyperlink ref="O15" r:id="rId5"/>
-    <hyperlink ref="O16" r:id="rId6"/>
-    <hyperlink ref="O17" r:id="rId7"/>
-    <hyperlink ref="O18" r:id="rId8"/>
-    <hyperlink ref="O19" r:id="rId9"/>
-    <hyperlink ref="O20" r:id="rId10"/>
-    <hyperlink ref="O21" r:id="rId11"/>
-    <hyperlink ref="O22" r:id="rId12"/>
-    <hyperlink ref="O10" r:id="rId13"/>
-    <hyperlink ref="O24" r:id="rId14"/>
-    <hyperlink ref="O25" r:id="rId15"/>
-    <hyperlink ref="O28" r:id="rId16"/>
-    <hyperlink ref="O29" r:id="rId17"/>
-    <hyperlink ref="O27" r:id="rId18"/>
-    <hyperlink ref="O23" r:id="rId19"/>
-    <hyperlink ref="O35" r:id="rId20"/>
-    <hyperlink ref="O38" r:id="rId21"/>
-    <hyperlink ref="O33" r:id="rId22"/>
-    <hyperlink ref="O34" r:id="rId23"/>
-    <hyperlink ref="O36" r:id="rId24"/>
-    <hyperlink ref="O37" r:id="rId25"/>
-    <hyperlink ref="O39" r:id="rId26"/>
-    <hyperlink ref="O40" r:id="rId27"/>
-    <hyperlink ref="O41" r:id="rId28"/>
-    <hyperlink ref="O42" r:id="rId29"/>
-    <hyperlink ref="O43" r:id="rId30"/>
-    <hyperlink ref="O45" r:id="rId31"/>
-    <hyperlink ref="O44" r:id="rId32"/>
-    <hyperlink ref="O46" r:id="rId33"/>
-    <hyperlink ref="O47" r:id="rId34"/>
-    <hyperlink ref="O48" r:id="rId35"/>
-    <hyperlink ref="O49" r:id="rId36"/>
-    <hyperlink ref="O50" r:id="rId37"/>
-    <hyperlink ref="O51" r:id="rId38"/>
-    <hyperlink ref="O52" r:id="rId39"/>
-    <hyperlink ref="O53" r:id="rId40"/>
-    <hyperlink ref="O55" r:id="rId41"/>
-    <hyperlink ref="O56" r:id="rId42"/>
-    <hyperlink ref="O57" r:id="rId43"/>
-    <hyperlink ref="O31" r:id="rId44"/>
-    <hyperlink ref="O30" r:id="rId45"/>
-    <hyperlink ref="O32" r:id="rId46"/>
-    <hyperlink ref="O54" r:id="rId47"/>
+    <hyperlink ref="O13" r:id="rId2"/>
+    <hyperlink ref="O14" r:id="rId3"/>
+    <hyperlink ref="O15" r:id="rId4"/>
+    <hyperlink ref="O16" r:id="rId5"/>
+    <hyperlink ref="O17" r:id="rId6"/>
+    <hyperlink ref="O18" r:id="rId7"/>
+    <hyperlink ref="O19" r:id="rId8"/>
+    <hyperlink ref="O20" r:id="rId9"/>
+    <hyperlink ref="O21" r:id="rId10"/>
+    <hyperlink ref="O22" r:id="rId11"/>
+    <hyperlink ref="O10" r:id="rId12"/>
+    <hyperlink ref="O24" r:id="rId13"/>
+    <hyperlink ref="O25" r:id="rId14"/>
+    <hyperlink ref="O28" r:id="rId15"/>
+    <hyperlink ref="O29" r:id="rId16"/>
+    <hyperlink ref="O27" r:id="rId17"/>
+    <hyperlink ref="O23" r:id="rId18"/>
+    <hyperlink ref="O35" r:id="rId19"/>
+    <hyperlink ref="O38" r:id="rId20"/>
+    <hyperlink ref="O33" r:id="rId21"/>
+    <hyperlink ref="O34" r:id="rId22"/>
+    <hyperlink ref="O36" r:id="rId23"/>
+    <hyperlink ref="O37" r:id="rId24"/>
+    <hyperlink ref="O39" r:id="rId25"/>
+    <hyperlink ref="O40" r:id="rId26"/>
+    <hyperlink ref="O41" r:id="rId27"/>
+    <hyperlink ref="O42" r:id="rId28"/>
+    <hyperlink ref="O43" r:id="rId29"/>
+    <hyperlink ref="O45" r:id="rId30"/>
+    <hyperlink ref="O44" r:id="rId31"/>
+    <hyperlink ref="O46" r:id="rId32"/>
+    <hyperlink ref="O47" r:id="rId33"/>
+    <hyperlink ref="O48" r:id="rId34"/>
+    <hyperlink ref="O49" r:id="rId35"/>
+    <hyperlink ref="O50" r:id="rId36"/>
+    <hyperlink ref="O51" r:id="rId37"/>
+    <hyperlink ref="O52" r:id="rId38"/>
+    <hyperlink ref="O53" r:id="rId39"/>
+    <hyperlink ref="O55" r:id="rId40"/>
+    <hyperlink ref="O56" r:id="rId41"/>
+    <hyperlink ref="O57" r:id="rId42"/>
+    <hyperlink ref="O31" r:id="rId43"/>
+    <hyperlink ref="O12" r:id="rId44"/>
+    <hyperlink ref="O32" r:id="rId45"/>
+    <hyperlink ref="O54" r:id="rId46"/>
+    <hyperlink ref="O30" r:id="rId47"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId48"/>

</xml_diff>